<commit_message>
Corrida | SFE-XMOI | 2026-06-17 11:55:41.088744
</commit_message>
<xml_diff>
--- a/indicadores/SFE-XMOI_out.xlsx
+++ b/indicadores/SFE-XMOI_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="442">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Exportaciones de MOI con origen en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Exportaciones de MOI</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">21/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1836,9 +1842,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1849,7 +1859,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1863,12 +1873,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.172065957784363</v>
+        <v>0.172212836065932</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1879,7 +1889,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1907,7 +1917,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1921,12 +1931,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.0286729105153152</v>
+        <v>0.0283257741576354</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1949,7 +1959,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1963,7 +1973,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1977,7 +1987,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1991,12 +2001,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.346433683564979</v>
+        <v>0.277463376819302</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2007,7 +2017,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2021,12 +2031,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.292122013070392</v>
+        <v>0.302784324557905</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2169,10 +2179,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2185,10 +2195,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2212,66 +2222,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>32.67753887</v>
@@ -2324,7 +2334,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>39.27598574</v>
@@ -2381,7 +2391,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>46.60720656</v>
@@ -2438,7 +2448,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>42.206922</v>
@@ -2495,7 +2505,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>50.49760772</v>
@@ -2552,7 +2562,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>48.871009</v>
@@ -2609,7 +2619,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>55.617589</v>
@@ -2666,7 +2676,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>56.792271</v>
@@ -2723,7 +2733,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>61.29915625</v>
@@ -2780,7 +2790,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>64.543266</v>
@@ -2837,7 +2847,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>55.21637</v>
@@ -2894,7 +2904,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>58.491764</v>
@@ -2951,7 +2961,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>43.60163465</v>
@@ -3010,7 +3020,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>52.025394</v>
@@ -3069,7 +3079,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>57.783019</v>
@@ -3128,7 +3138,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>54.26334826</v>
@@ -3187,7 +3197,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>55.998136</v>
@@ -3246,7 +3256,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>52.453692</v>
@@ -3305,7 +3315,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>57.00102969</v>
@@ -3364,7 +3374,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>55.37735862</v>
@@ -3423,7 +3433,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>59.04863854</v>
@@ -3482,7 +3492,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>62.15918564</v>
@@ -3541,7 +3551,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>61.348637</v>
@@ -3600,7 +3610,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>58.99751974</v>
@@ -3659,7 +3669,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>53.8348352</v>
@@ -3718,7 +3728,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>50.26878139</v>
@@ -3777,7 +3787,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>68.72892562</v>
@@ -3836,7 +3846,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>48.71114262</v>
@@ -3895,7 +3905,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>76.18205319</v>
@@ -3954,7 +3964,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>60.90251996</v>
@@ -4013,7 +4023,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>65.42236158</v>
@@ -4072,7 +4082,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>75.54145127</v>
@@ -4131,7 +4141,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>71.5945105</v>
@@ -4190,7 +4200,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>90.22980678</v>
@@ -4249,7 +4259,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>101.31022789</v>
@@ -4308,7 +4318,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>114.62555936</v>
@@ -4367,7 +4377,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>71.66903919</v>
@@ -4426,7 +4436,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>73.13478447</v>
@@ -4485,7 +4495,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>80.11710725</v>
@@ -4544,7 +4554,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>83.20158344</v>
@@ -4603,7 +4613,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>82.31429798</v>
@@ -4662,7 +4672,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>71.75006513</v>
@@ -4721,7 +4731,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>75.38904716</v>
@@ -4780,7 +4790,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>84.06034524</v>
@@ -4839,7 +4849,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>78.73760137</v>
@@ -4898,7 +4908,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>87.16245433</v>
@@ -4957,7 +4967,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>90.87630647</v>
@@ -5016,7 +5026,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>85.87825189</v>
@@ -5075,7 +5085,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>54.25794894</v>
@@ -5134,7 +5144,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>64.9546609</v>
@@ -5193,7 +5203,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>81.31320061</v>
@@ -5252,7 +5262,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>77.37584733</v>
@@ -5311,7 +5321,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>94.39892642</v>
@@ -5370,7 +5380,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>92.13632759</v>
@@ -5429,7 +5439,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>83.71014769</v>
@@ -5488,7 +5498,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>99.09698182</v>
@@ -5547,7 +5557,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>113.47509261</v>
@@ -5606,7 +5616,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>88.96455486</v>
@@ -5665,7 +5675,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>127.09024933</v>
@@ -5724,7 +5734,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>119.83745175</v>
@@ -5783,7 +5793,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>77.50610694</v>
@@ -5842,7 +5852,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>108.08011543</v>
@@ -5901,7 +5911,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>118.7714098</v>
@@ -5960,7 +5970,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>106.62149123</v>
@@ -6019,7 +6029,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>110.42875023</v>
@@ -6078,7 +6088,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>138.84949975</v>
@@ -6137,7 +6147,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>131.67952586</v>
@@ -6196,7 +6206,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>138.51141617</v>
@@ -6255,7 +6265,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>152.45987111</v>
@@ -6314,7 +6324,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>156.47792227</v>
@@ -6373,7 +6383,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>170.82083905</v>
@@ -6432,7 +6442,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>162.69085573</v>
@@ -6491,7 +6501,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>115.77859983</v>
@@ -6550,7 +6560,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>117.86687568</v>
@@ -6609,7 +6619,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>136.86309182</v>
@@ -6668,7 +6678,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>138.38399927</v>
@@ -6727,7 +6737,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>149.56069798</v>
@@ -6786,7 +6796,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>141.08488603</v>
@@ -6845,7 +6855,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>181.77838038</v>
@@ -6904,7 +6914,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>206.69234472</v>
@@ -6963,7 +6973,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>258.65697593</v>
@@ -7022,7 +7032,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>215.93881401</v>
@@ -7081,7 +7091,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>137.89329094</v>
@@ -7140,7 +7150,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>129.65169708</v>
@@ -7199,7 +7209,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>87.72206082</v>
@@ -7258,7 +7268,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>88.58955279</v>
@@ -7317,7 +7327,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>133.40298047</v>
@@ -7376,7 +7386,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>128.5548491</v>
@@ -7435,7 +7445,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>144.34289789</v>
@@ -7494,7 +7504,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>156.98364364</v>
@@ -7553,7 +7563,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>193.14928662</v>
@@ -7612,7 +7622,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>172.68056778</v>
@@ -7671,7 +7681,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>202.0671402</v>
@@ -7730,7 +7740,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>214.9346741</v>
@@ -7789,7 +7799,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>246.27212888</v>
@@ -7848,7 +7858,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>245.29147717</v>
@@ -7907,7 +7917,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>227.13696605</v>
@@ -7966,7 +7976,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>224.99474831</v>
@@ -8025,7 +8035,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>189.45269179</v>
@@ -8084,7 +8094,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>203.53028696</v>
@@ -8143,7 +8153,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>222.65665022</v>
@@ -8202,7 +8212,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>266.05280033</v>
@@ -8261,7 +8271,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>223.77374103</v>
@@ -8320,7 +8330,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>287.01346596</v>
@@ -8379,7 +8389,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>272.0171243</v>
@@ -8438,7 +8448,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>304.66657041</v>
@@ -8497,7 +8507,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>269.23110734</v>
@@ -8556,7 +8566,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>309.23535452</v>
@@ -8615,7 +8625,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>306.14365938</v>
@@ -8674,7 +8684,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>268.03403136</v>
@@ -8733,7 +8743,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>286.44521589</v>
@@ -8792,7 +8802,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>310.96819574</v>
@@ -8851,7 +8861,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>351.55942114</v>
@@ -8910,7 +8920,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>350.96544992</v>
@@ -8969,7 +8979,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>392.87512325</v>
@@ -9028,7 +9038,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>370.69912886</v>
@@ -9087,7 +9097,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>366.13886572</v>
@@ -9146,7 +9156,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>395.04330521</v>
@@ -9205,7 +9215,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>328.72057886</v>
@@ -9264,7 +9274,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>390.70400406</v>
@@ -9323,7 +9333,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>333.79468365</v>
@@ -9382,7 +9392,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>297.84421131</v>
@@ -9441,7 +9451,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>367.45353728</v>
@@ -9500,7 +9510,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>385.47576509</v>
@@ -9559,7 +9569,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>265.19547063</v>
@@ -9618,7 +9628,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>397.52469924</v>
@@ -9677,7 +9687,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>329.80824636</v>
@@ -9736,7 +9746,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>354.766854</v>
@@ -9795,7 +9805,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>262.82404859</v>
@@ -9854,7 +9864,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>247.49910671</v>
@@ -9913,7 +9923,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>245.47888326</v>
@@ -9972,7 +9982,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>305.3995273</v>
@@ -10031,7 +10041,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>250.12133282</v>
@@ -10090,7 +10100,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>174.54783675</v>
@@ -10149,7 +10159,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>204.8680545</v>
@@ -10208,7 +10218,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>227.41742177</v>
@@ -10267,7 +10277,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>214.81177884</v>
@@ -10326,7 +10336,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>263.95239054</v>
@@ -10385,7 +10395,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>212.88041395</v>
@@ -10444,7 +10454,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>294.73460815</v>
@@ -10503,7 +10513,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>263.56087309</v>
@@ -10562,7 +10572,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>334.41884396</v>
@@ -10621,7 +10631,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>315.18690431</v>
@@ -10680,7 +10690,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>192.04162997</v>
@@ -10739,7 +10749,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>122.5361685</v>
@@ -10798,7 +10808,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>153.96577335</v>
@@ -10857,7 +10867,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>214.17993297</v>
@@ -10916,7 +10926,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>178.73440629</v>
@@ -10975,7 +10985,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>243.7752898</v>
@@ -11034,7 +11044,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>219.42565298</v>
@@ -11093,7 +11103,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>266.50152764</v>
@@ -11152,7 +11162,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>284.62940479</v>
@@ -11211,7 +11221,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>268.88728228</v>
@@ -11270,7 +11280,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>296.08264944</v>
@@ -11329,7 +11339,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>206.77153255</v>
@@ -11388,7 +11398,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>197.03617562</v>
@@ -11447,7 +11457,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>75.77802932</v>
@@ -11506,7 +11516,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>100.60659792</v>
@@ -11565,7 +11575,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>133.78878075</v>
@@ -11624,7 +11634,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>96.62323535</v>
@@ -11683,7 +11693,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>98.80664607</v>
@@ -11742,7 +11752,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>129.71083435</v>
@@ -11801,7 +11811,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>119.76912341</v>
@@ -11860,7 +11870,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>141.50789805</v>
@@ -11919,7 +11929,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>133.71260863</v>
@@ -11978,7 +11988,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>120.03281887</v>
@@ -12037,7 +12047,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>150.14962225</v>
@@ -12096,7 +12106,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>83.6651228</v>
@@ -12155,7 +12165,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>70.77635787</v>
@@ -12214,7 +12224,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>82.16566348</v>
@@ -12273,7 +12283,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>123.12226222</v>
@@ -12332,7 +12342,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>117.75028896</v>
@@ -12391,7 +12401,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>174.0393255</v>
@@ -12450,7 +12460,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>200.02986255</v>
@@ -12509,7 +12519,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>187.22356503</v>
@@ -12568,7 +12578,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>216.69914854</v>
@@ -12627,7 +12637,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>230.33063538</v>
@@ -12686,7 +12696,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>260.64134858</v>
@@ -12745,7 +12755,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>220.63225754</v>
@@ -12804,7 +12814,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>197.93770159</v>
@@ -12863,7 +12873,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>128.01074384</v>
@@ -12922,7 +12932,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>129.52332666</v>
@@ -12981,7 +12991,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>94.88707132</v>
@@ -13040,7 +13050,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>205.95342192</v>
@@ -13099,7 +13109,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>251.68940605</v>
@@ -13158,7 +13168,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>234.46997297</v>
@@ -13217,7 +13227,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>242.13074185</v>
@@ -13276,7 +13286,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>178.21775444</v>
@@ -13335,7 +13345,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>177.44077446</v>
@@ -13394,7 +13404,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>232.45485354</v>
@@ -13453,7 +13463,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>225.01843164</v>
@@ -13512,7 +13522,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>245.06154607</v>
@@ -13571,7 +13581,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>181.11843122</v>
@@ -13630,7 +13640,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>149.85677833</v>
@@ -13689,7 +13699,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>149.48695949</v>
@@ -13748,7 +13758,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>173.87437122</v>
@@ -13807,7 +13817,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>172.60741184</v>
@@ -13866,7 +13876,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>285.555274</v>
@@ -13925,7 +13935,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>288.78919951</v>
@@ -13984,7 +13994,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>188.49364821</v>
@@ -14043,7 +14053,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>153.26597597</v>
@@ -14102,7 +14112,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>116.9634744</v>
@@ -14161,7 +14171,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>224.37628861</v>
@@ -14220,7 +14230,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>180.4230966</v>
@@ -14279,7 +14289,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>74.04698944</v>
@@ -14338,7 +14348,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>98.29430427</v>
@@ -14397,7 +14407,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>159.35516911</v>
@@ -14456,7 +14466,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>198.03653504</v>
@@ -14515,7 +14525,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>241.44535009</v>
@@ -14574,7 +14584,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>148.25113044</v>
@@ -14633,7 +14643,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>184.76485996</v>
@@ -14692,7 +14702,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>153.15806443</v>
@@ -14751,7 +14761,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>202.04169506</v>
@@ -14810,7 +14820,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>89.79259641</v>
@@ -14869,7 +14879,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>158.87288862</v>
@@ -14928,7 +14938,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>217.90536678</v>
@@ -14987,7 +14997,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>79.26159886</v>
@@ -15046,7 +15056,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>100.78143058</v>
@@ -15105,7 +15115,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>180.92791797</v>
@@ -15164,7 +15174,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>66.84228967</v>
@@ -15223,7 +15233,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>47.71904343</v>
@@ -15282,7 +15292,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>63.913774</v>
@@ -15341,7 +15351,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>131.56461383</v>
@@ -15400,7 +15410,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>101.6483794</v>
@@ -15459,7 +15469,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>169.68801746</v>
@@ -15518,7 +15528,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>74.7445238</v>
@@ -15577,7 +15587,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>77.94224519</v>
@@ -15636,7 +15646,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>64.12599604</v>
@@ -15695,7 +15705,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>116.60746111</v>
@@ -15754,7 +15764,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>144.40233257</v>
@@ -15813,7 +15823,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>179.57574331</v>
@@ -15872,7 +15882,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>92.31727213</v>
@@ -15931,7 +15941,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>219.52910256</v>
@@ -15990,7 +16000,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>260.65459324</v>
@@ -16049,7 +16059,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>325.91625389</v>
@@ -16108,7 +16118,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>243.35407851</v>
@@ -16167,7 +16177,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>228.76807054</v>
@@ -16226,7 +16236,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>276.48136998</v>
@@ -16285,7 +16295,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>145.10305226</v>
@@ -16344,7 +16354,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>104.9113459</v>
@@ -16403,7 +16413,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>239.61414961</v>
@@ -16462,7 +16472,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>257.25267499</v>
@@ -16521,7 +16531,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>276.25757924</v>
@@ -16580,7 +16590,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>269.45294816</v>
@@ -16639,7 +16649,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>257.58286975</v>
@@ -16698,7 +16708,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>330.88315893</v>
@@ -16757,7 +16767,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>170.54694615</v>
@@ -16816,7 +16826,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>167.34025198</v>
@@ -16875,7 +16885,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>162.87149766</v>
@@ -16934,7 +16944,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>246.25542005</v>
@@ -16993,7 +17003,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>281.86990469</v>
@@ -17052,7 +17062,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>192.02827332</v>
@@ -17111,7 +17121,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>107.54664481</v>
@@ -17170,7 +17180,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>104.38965983</v>
@@ -17229,7 +17239,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>124.33460092</v>
@@ -17288,7 +17298,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>198.20598565</v>
@@ -17347,7 +17357,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>125.84065174</v>
@@ -17406,7 +17416,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>108.56841477</v>
@@ -17465,7 +17475,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>126.442929</v>
@@ -17524,7 +17534,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>140.17291838</v>
@@ -17583,7 +17593,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>138.03613472</v>
@@ -17642,7 +17652,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>128.15329743</v>
@@ -17701,7 +17711,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>95.98927091</v>
@@ -17760,7 +17770,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>56.37402781</v>
@@ -17819,7 +17829,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>53.86657217</v>
@@ -17878,7 +17888,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>57.67325974</v>
@@ -17937,7 +17947,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>75.60246236</v>
@@ -17996,7 +18006,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>118.80312224</v>
@@ -18055,7 +18065,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>151.53957798</v>
@@ -18114,7 +18124,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>120.79839631</v>
@@ -18173,7 +18183,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>160.09897204</v>
@@ -18232,7 +18242,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>152.33647799</v>
@@ -18291,7 +18301,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>146.5777621</v>
@@ -18350,7 +18360,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>141.30641128</v>
@@ -18409,7 +18419,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>165.91168039</v>
@@ -18468,7 +18478,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>179.66377143</v>
@@ -18527,7 +18537,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>76.47253625</v>
@@ -18586,7 +18596,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>126.93828362</v>
@@ -18645,7 +18655,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>132.83633323</v>
@@ -18704,7 +18714,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>82.79595765</v>
@@ -18763,7 +18773,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>131.06510337</v>
@@ -18822,7 +18832,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>73.44548019</v>
@@ -18881,7 +18891,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>130.29198121</v>
@@ -18940,7 +18950,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>186.78534634</v>
@@ -18999,7 +19009,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>147.53700855</v>
@@ -19058,7 +19068,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>157.19853319</v>
@@ -19117,7 +19127,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>137.5254458</v>
@@ -19176,7 +19186,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>117.23127629</v>
@@ -19235,7 +19245,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>62.62020002</v>
@@ -19294,7 +19304,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>102.24898882</v>
@@ -19353,7 +19363,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>118.20557839</v>
@@ -19412,7 +19422,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>102.77960343</v>
@@ -19471,7 +19481,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2"/>
       <c r="C294" s="3" t="n">
@@ -19504,7 +19514,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2"/>
       <c r="C295" s="3" t="n">
@@ -19537,7 +19547,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2"/>
       <c r="C296" s="3" t="n">
@@ -19570,7 +19580,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2"/>
       <c r="C297" s="3" t="n">
@@ -19603,7 +19613,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2"/>
       <c r="C298" s="3" t="n">
@@ -19636,7 +19646,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2"/>
       <c r="C299" s="3" t="n">
@@ -19669,7 +19679,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2"/>
       <c r="C300" s="3" t="n">
@@ -19702,7 +19712,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2"/>
       <c r="C301" s="3" t="n">
@@ -19735,7 +19745,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2"/>
       <c r="C302" s="3" t="n">
@@ -19768,7 +19778,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2"/>
       <c r="C303" s="3" t="n">
@@ -19801,7 +19811,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2"/>
       <c r="C304" s="3" t="n">
@@ -19834,7 +19844,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2"/>
       <c r="C305" s="3" t="n">
@@ -19867,7 +19877,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2"/>
       <c r="C306" s="3"/>
@@ -19890,7 +19900,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2"/>
       <c r="C307" s="3"/>
@@ -19913,7 +19923,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2"/>
       <c r="C308" s="3"/>
@@ -19936,7 +19946,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2"/>
       <c r="C309" s="3"/>
@@ -19959,7 +19969,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2"/>
       <c r="C310" s="3"/>
@@ -19982,7 +19992,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2"/>
       <c r="C311" s="3"/>
@@ -20005,7 +20015,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2"/>
       <c r="C312" s="3"/>
@@ -20028,7 +20038,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2"/>
       <c r="C313" s="3"/>
@@ -20051,7 +20061,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2"/>
       <c r="C314" s="3"/>
@@ -20074,7 +20084,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2"/>
       <c r="C315" s="3"/>
@@ -20097,7 +20107,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2"/>
       <c r="C316" s="3"/>
@@ -20120,7 +20130,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2"/>
       <c r="C317" s="3"/>
@@ -20143,7 +20153,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2"/>
       <c r="C318" s="3"/>
@@ -20166,7 +20176,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2"/>
       <c r="C319" s="3"/>
@@ -20189,7 +20199,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2"/>
       <c r="C320" s="3"/>
@@ -20212,7 +20222,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2"/>
       <c r="C321" s="3"/>
@@ -20235,7 +20245,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="3"/>
@@ -20258,7 +20268,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2"/>
       <c r="C323" s="3"/>
@@ -20281,7 +20291,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2"/>
       <c r="C324" s="3"/>
@@ -20304,7 +20314,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2"/>
       <c r="C325" s="3"/>
@@ -20327,7 +20337,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2"/>
       <c r="C326" s="3"/>
@@ -20350,7 +20360,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2"/>
       <c r="C327" s="3"/>
@@ -20373,7 +20383,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2"/>
       <c r="C328" s="3"/>
@@ -20396,7 +20406,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2"/>
       <c r="C329" s="3"/>
@@ -20419,7 +20429,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2"/>
       <c r="C330" s="3"/>
@@ -20442,7 +20452,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2"/>
       <c r="C331" s="3"/>
@@ -20465,7 +20475,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2"/>
       <c r="C332" s="3"/>
@@ -20488,7 +20498,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2"/>
       <c r="C333" s="3"/>
@@ -20511,7 +20521,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2"/>
       <c r="C334" s="3"/>
@@ -20534,7 +20544,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2"/>
       <c r="C335" s="3"/>
@@ -20557,7 +20567,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2"/>
       <c r="C336" s="3"/>
@@ -20580,7 +20590,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2"/>
       <c r="C337" s="3"/>
@@ -20603,7 +20613,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2"/>
       <c r="C338" s="3"/>
@@ -20626,7 +20636,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2"/>
       <c r="C339" s="3"/>
@@ -20649,7 +20659,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2"/>
       <c r="C340" s="3"/>
@@ -20672,7 +20682,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2"/>
       <c r="C341" s="3"/>
@@ -20695,7 +20705,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2"/>
       <c r="C342" s="3"/>
@@ -20718,7 +20728,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2"/>
       <c r="C343" s="3"/>
@@ -20741,7 +20751,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2"/>
       <c r="C344" s="3"/>
@@ -20764,7 +20774,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2"/>
       <c r="C345" s="3"/>
@@ -20787,7 +20797,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2"/>
       <c r="C346" s="3"/>
@@ -20810,7 +20820,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2"/>
       <c r="C347" s="3"/>
@@ -20833,7 +20843,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2"/>
       <c r="C348" s="3"/>
@@ -20856,7 +20866,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2"/>
       <c r="C349" s="3"/>
@@ -20890,97 +20900,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -21004,7 +21014,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -21014,160 +21024,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.128144001483692</v>
+        <v>0.13081294689564</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.141742526454879</v>
+        <v>0.144570141376814</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0720848486165068</v>
+        <v>0.0719185100120539</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>-0.00353583222961168</v>
+        <v>-0.00463180437836369</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.0168416366514499</v>
+        <v>-0.0168014781272174</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.0441617641859748</v>
+        <v>0.0449411020162555</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.136034293082452</v>
+        <v>0.136002750912079</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.172065957784363</v>
+        <v>0.172212836065932</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.161039894475264</v>
+        <v>0.160820070676705</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.169330772499611</v>
+        <v>0.168302626710445</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.149959617998544</v>
+        <v>0.149360617462258</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.0785459683137238</v>
+        <v>0.0784290104312591</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.0150276456031417</v>
+        <v>0.0155971144969826</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.00768183099656496</v>
+        <v>0.00921653051918652</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0440920803532682</v>
+        <v>0.0467113576590665</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0956513945871116</v>
+        <v>0.0974544686572482</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.0924824742268859</v>
+        <v>0.0916250377383199</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.023165132732983</v>
+        <v>0.0208797632448223</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.01324203773091</v>
+        <v>-0.0142883339151938</v>
       </c>
     </row>
     <row r="24">

</xml_diff>